<commit_message>
Suggest the user from the room, pick school users, drop "Khu vực"
- Nhập mới: Nơi sử dụng and Người sử dụng sit outside the form, so
  choosing a room immediately suggests its user (most common user of
  equipment in that room, else the room manager).
- A shared user picker (type to search, or enter a new email) lists
  SharePoint site users with names (bridge mode) plus users known from
  roles, room managers and equipment; used on Nhập mới, Chỉnh sửa,
  Điều chuyển and when adding a room. Emails are lower-cased, names kept.
- Room labels no longer repeat the code when the room name equals it
  ("Ham_Bep - Ham_Bep" -> "Ham_Bep").
- Removed the "Khu vực" column from the room list everywhere (schema,
  room page, templates, demo data, README).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWuJVkZ8QmJV6ZRpzrxWrn
</commit_message>
<xml_diff>
--- a/templates/2_Phong.xlsx
+++ b/templates/2_Phong.xlsx
@@ -144,14 +144,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_Phong" displayName="tbl_Phong" ref="A1:E2" headerRowCount="1">
-  <autoFilter ref="A1:E2"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_Phong" displayName="tbl_Phong" ref="A1:D2" headerRowCount="1">
+  <autoFilter ref="A1:D2"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="Mã phòng"/>
     <tableColumn id="2" name="Tên phòng"/>
-    <tableColumn id="3" name="Khu vực"/>
-    <tableColumn id="4" name="Email người quản lý"/>
-    <tableColumn id="5" name="Tên người quản lý"/>
+    <tableColumn id="3" name="Email người quản lý"/>
+    <tableColumn id="4" name="Tên người quản lý"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -446,14 +445,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,15 +467,10 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Khu vực</t>
+          <t>Email người quản lý</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>Email người quản lý</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>Tên người quản lý</t>
         </is>
@@ -496,15 +489,10 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tầng trệt</t>
+          <t>giaovien@truong.edu.vn</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>giaovien@truong.edu.vn</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>Nguyễn Văn A</t>
         </is>
@@ -524,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -599,7 +587,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Khu vực</t>
+          <t>Email người quản lý</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -612,7 +600,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Email người quản lý</t>
+          <t>Tên người quản lý</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -621,19 +609,6 @@
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tên người quản lý</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Một dòng văn bản (Single line of text)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>